<commit_message>
Updating final exam notebook and data
</commit_message>
<xml_diff>
--- a/Assignments/Final-Exam/Busters Burrito Sales.xlsx
+++ b/Assignments/Final-Exam/Busters Burrito Sales.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>767.87</v>
+        <v>800.9299999999999</v>
       </c>
     </row>
     <row r="3">
@@ -413,13 +413,13 @@
         </is>
       </c>
       <c r="D3">
-        <v>875.14</v>
+        <v>895.4400000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Brewery</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -433,7 +433,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>865.84</v>
+        <v>728.4400000000001</v>
       </c>
     </row>
     <row r="5">
@@ -453,18 +453,18 @@
         </is>
       </c>
       <c r="D5">
-        <v>544.24</v>
+        <v>739.61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Brewery</t>
+          <t>University</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Weekend</t>
+          <t>Weekday</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -473,18 +473,18 @@
         </is>
       </c>
       <c r="D6">
-        <v>1055.34</v>
+        <v>804.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brewery</t>
+          <t>University</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Weekend</t>
+          <t>Weekday</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="D7">
-        <v>1211.47</v>
+        <v>660.46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Brewery</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -513,13 +513,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>1107.86</v>
+        <v>1272.87</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Brewery</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>989.51</v>
+        <v>1221.42</v>
       </c>
     </row>
     <row r="10">
@@ -544,36 +544,36 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>Weekend</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Partnership</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="D10">
-        <v>1080</v>
+        <v>1193.33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Brewery</t>
+          <t>University</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>Weekend</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Partnership</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="D11">
-        <v>1089.29</v>
+        <v>1102.79</v>
       </c>
     </row>
     <row r="12">
@@ -584,16 +584,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>Weekend</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Partnership</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="D12">
-        <v>910.1799999999999</v>
+        <v>966.96</v>
       </c>
     </row>
     <row r="13">
@@ -604,16 +604,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Weekday</t>
+          <t>Weekend</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Partnership</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="D13">
-        <v>894.61</v>
+        <v>1089.46</v>
       </c>
     </row>
     <row r="14">
@@ -624,7 +624,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Weekend</t>
+          <t>Weekday</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>1361.9</v>
+        <v>1033.87</v>
       </c>
     </row>
     <row r="15">
@@ -644,7 +644,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Weekend</t>
+          <t>Weekday</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -653,18 +653,18 @@
         </is>
       </c>
       <c r="D15">
-        <v>1428.39</v>
+        <v>1115.93</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Brewery</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Weekend</t>
+          <t>Weekday</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>1262.99</v>
+        <v>1047.1</v>
       </c>
     </row>
     <row r="17">
@@ -684,7 +684,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Weekend</t>
+          <t>Weekday</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -693,7 +693,167 @@
         </is>
       </c>
       <c r="D17">
-        <v>1357.65</v>
+        <v>829.45</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Weekday</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D18">
+        <v>813.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Weekday</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D19">
+        <v>814.83</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brewery</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Weekend</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D20">
+        <v>1352.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Brewery</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Weekend</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D21">
+        <v>1492.71</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Brewery</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Weekend</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D22">
+        <v>1415.29</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Weekend</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D23">
+        <v>1281.94</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Weekend</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D24">
+        <v>1163.42</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Weekend</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="D25">
+        <v>1362.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>